<commit_message>
Spreadsheet: defined names and conditional formatting
Names (Insert > Names, or typed in the Name Box for the selection): formulas
name ranges and values; shifted with the rows and columns; read and written in
.xlsx, read from .ods. Conditional formatting (Format > Conditional Formatting):
cell value, text, top / bottom, average, duplicates, formula rules with their
looks, colour scales, data bars; read and written in .xlsx (dxfs), read from
LibreOffice's .ods. The sample workbook shows both; tests through LibreOffice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HNkQXkWmCNHsSExBnbTMLo
</commit_message>
<xml_diff>
--- a/sdcard/docs/cafe-2026.xlsx
+++ b/sdcard/docs/cafe-2026.xlsx
@@ -10,6 +10,11 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
     <sheet name="Loan" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="Amount">Loan!$B$3</definedName>
+    <definedName name="Rate">Loan!$B$4</definedName>
+    <definedName name="Months">Loan!$B$5</definedName>
+  </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -311,6 +316,19 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -1042,6 +1060,18 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
   </mergeCells>
+  <conditionalFormatting sqref="E5:E16">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF6FA8DC"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:B16">
+    <cfRule type="top10" dxfId="0" priority="2" rank="3"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -1239,7 +1269,7 @@
         <v>24</v>
       </c>
       <c r="B6" s="5">
-        <f>PMT(B4/12,B5,-B3)</f>
+        <f>PMT(Rate/12,Months,-Amount)</f>
         <v>356.96309374051395</v>
       </c>
     </row>
@@ -1248,7 +1278,7 @@
         <v>25</v>
       </c>
       <c r="B7" s="12">
-        <f>B6*B5-B3</f>
+        <f>B6*Months-Amount</f>
         <v>850.67137465850283</v>
       </c>
     </row>
@@ -1278,15 +1308,15 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C10" s="12">
-        <f>IPMT($B$4/12,A10,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A10,Months,-Amount)</f>
         <v>45</v>
       </c>
       <c r="D10" s="12">
-        <f>PPMT($B$4/12,A10,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A10,Months,-Amount)</f>
         <v>311.96309374051395</v>
       </c>
       <c r="E10" s="12">
-        <f>$B$3-D10</f>
+        <f>Amount-D10</f>
         <v>11688.036906259485</v>
       </c>
     </row>
@@ -1299,11 +1329,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C11" s="8">
-        <f>IPMT($B$4/12,A11,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A11,Months,-Amount)</f>
         <v>43.830138398473089</v>
       </c>
       <c r="D11" s="8">
-        <f>PPMT($B$4/12,A11,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A11,Months,-Amount)</f>
         <v>313.13295534204087</v>
       </c>
       <c r="E11" s="8">
@@ -1320,11 +1350,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C12" s="12">
-        <f>IPMT($B$4/12,A12,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A12,Months,-Amount)</f>
         <v>42.655889815940462</v>
       </c>
       <c r="D12" s="12">
-        <f>PPMT($B$4/12,A12,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A12,Months,-Amount)</f>
         <v>314.30720392457351</v>
       </c>
       <c r="E12" s="12">
@@ -1341,11 +1371,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C13" s="8">
-        <f>IPMT($B$4/12,A13,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A13,Months,-Amount)</f>
         <v>41.477237801223367</v>
       </c>
       <c r="D13" s="8">
-        <f>PPMT($B$4/12,A13,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A13,Months,-Amount)</f>
         <v>315.48585593929056</v>
       </c>
       <c r="E13" s="8">
@@ -1362,11 +1392,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C14" s="12">
-        <f>IPMT($B$4/12,A14,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A14,Months,-Amount)</f>
         <v>40.294165841451033</v>
       </c>
       <c r="D14" s="12">
-        <f>PPMT($B$4/12,A14,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A14,Months,-Amount)</f>
         <v>316.66892789906291</v>
       </c>
       <c r="E14" s="12">
@@ -1383,11 +1413,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C15" s="8">
-        <f>IPMT($B$4/12,A15,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A15,Months,-Amount)</f>
         <v>39.106657361829555</v>
       </c>
       <c r="D15" s="8">
-        <f>PPMT($B$4/12,A15,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A15,Months,-Amount)</f>
         <v>317.85643637868441</v>
       </c>
       <c r="E15" s="8">
@@ -1404,11 +1434,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C16" s="12">
-        <f>IPMT($B$4/12,A16,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A16,Months,-Amount)</f>
         <v>37.914695725409516</v>
       </c>
       <c r="D16" s="12">
-        <f>PPMT($B$4/12,A16,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A16,Months,-Amount)</f>
         <v>319.04839801510445</v>
       </c>
       <c r="E16" s="12">
@@ -1425,11 +1455,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C17" s="8">
-        <f>IPMT($B$4/12,A17,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A17,Months,-Amount)</f>
         <v>36.718264232852931</v>
       </c>
       <c r="D17" s="8">
-        <f>PPMT($B$4/12,A17,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A17,Months,-Amount)</f>
         <v>320.24482950766105</v>
       </c>
       <c r="E17" s="8">
@@ -1446,11 +1476,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C18" s="12">
-        <f>IPMT($B$4/12,A18,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A18,Months,-Amount)</f>
         <v>35.5173461221992</v>
       </c>
       <c r="D18" s="12">
-        <f>PPMT($B$4/12,A18,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A18,Months,-Amount)</f>
         <v>321.44574761831473</v>
       </c>
       <c r="E18" s="12">
@@ -1467,11 +1497,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C19" s="8">
-        <f>IPMT($B$4/12,A19,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A19,Months,-Amount)</f>
         <v>34.311924568630523</v>
       </c>
       <c r="D19" s="8">
-        <f>PPMT($B$4/12,A19,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A19,Months,-Amount)</f>
         <v>322.65116917188345</v>
       </c>
       <c r="E19" s="8">
@@ -1488,11 +1518,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C20" s="12">
-        <f>IPMT($B$4/12,A20,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A20,Months,-Amount)</f>
         <v>33.101982684236013</v>
       </c>
       <c r="D20" s="12">
-        <f>PPMT($B$4/12,A20,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A20,Months,-Amount)</f>
         <v>323.86111105627793</v>
       </c>
       <c r="E20" s="12">
@@ -1509,11 +1539,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C21" s="8">
-        <f>IPMT($B$4/12,A21,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A21,Months,-Amount)</f>
         <v>31.887503517775002</v>
       </c>
       <c r="D21" s="8">
-        <f>PPMT($B$4/12,A21,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A21,Months,-Amount)</f>
         <v>325.07559022273892</v>
       </c>
       <c r="E21" s="8">
@@ -1530,11 +1560,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C22" s="12">
-        <f>IPMT($B$4/12,A22,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A22,Months,-Amount)</f>
         <v>30.668470054439744</v>
       </c>
       <c r="D22" s="12">
-        <f>PPMT($B$4/12,A22,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A22,Months,-Amount)</f>
         <v>326.2946236860742</v>
       </c>
       <c r="E22" s="12">
@@ -1551,11 +1581,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C23" s="8">
-        <f>IPMT($B$4/12,A23,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A23,Months,-Amount)</f>
         <v>29.444865215617018</v>
       </c>
       <c r="D23" s="8">
-        <f>PPMT($B$4/12,A23,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A23,Months,-Amount)</f>
         <v>327.51822852489693</v>
       </c>
       <c r="E23" s="8">
@@ -1572,11 +1602,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C24" s="12">
-        <f>IPMT($B$4/12,A24,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A24,Months,-Amount)</f>
         <v>28.21667185864866</v>
       </c>
       <c r="D24" s="12">
-        <f>PPMT($B$4/12,A24,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A24,Months,-Amount)</f>
         <v>328.74642188186527</v>
       </c>
       <c r="E24" s="12">
@@ -1593,11 +1623,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C25" s="8">
-        <f>IPMT($B$4/12,A25,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A25,Months,-Amount)</f>
         <v>26.983872776591674</v>
       </c>
       <c r="D25" s="8">
-        <f>PPMT($B$4/12,A25,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A25,Months,-Amount)</f>
         <v>329.97922096392227</v>
       </c>
       <c r="E25" s="8">
@@ -1614,11 +1644,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C26" s="12">
-        <f>IPMT($B$4/12,A26,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A26,Months,-Amount)</f>
         <v>25.746450697977011</v>
       </c>
       <c r="D26" s="12">
-        <f>PPMT($B$4/12,A26,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A26,Months,-Amount)</f>
         <v>331.21664304253693</v>
       </c>
       <c r="E26" s="12">
@@ -1635,11 +1665,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C27" s="8">
-        <f>IPMT($B$4/12,A27,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A27,Months,-Amount)</f>
         <v>24.504388286567544</v>
       </c>
       <c r="D27" s="8">
-        <f>PPMT($B$4/12,A27,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A27,Months,-Amount)</f>
         <v>332.45870545394644</v>
       </c>
       <c r="E27" s="8">
@@ -1656,11 +1686,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C28" s="12">
-        <f>IPMT($B$4/12,A28,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A28,Months,-Amount)</f>
         <v>23.257668141115253</v>
       </c>
       <c r="D28" s="12">
-        <f>PPMT($B$4/12,A28,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A28,Months,-Amount)</f>
         <v>333.70542559939872</v>
       </c>
       <c r="E28" s="12">
@@ -1677,11 +1707,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C29" s="8">
-        <f>IPMT($B$4/12,A29,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A29,Months,-Amount)</f>
         <v>22.006272795117553</v>
       </c>
       <c r="D29" s="8">
-        <f>PPMT($B$4/12,A29,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A29,Months,-Amount)</f>
         <v>334.95682094539643</v>
       </c>
       <c r="E29" s="8">
@@ -1698,11 +1728,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C30" s="12">
-        <f>IPMT($B$4/12,A30,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A30,Months,-Amount)</f>
         <v>20.750184716572342</v>
       </c>
       <c r="D30" s="12">
-        <f>PPMT($B$4/12,A30,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A30,Months,-Amount)</f>
         <v>336.21290902394162</v>
       </c>
       <c r="E30" s="12">
@@ -1719,11 +1749,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C31" s="8">
-        <f>IPMT($B$4/12,A31,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A31,Months,-Amount)</f>
         <v>19.489386307732595</v>
       </c>
       <c r="D31" s="8">
-        <f>PPMT($B$4/12,A31,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A31,Months,-Amount)</f>
         <v>337.47370743278134</v>
       </c>
       <c r="E31" s="8">
@@ -1740,11 +1770,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C32" s="12">
-        <f>IPMT($B$4/12,A32,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A32,Months,-Amount)</f>
         <v>18.22385990485968</v>
       </c>
       <c r="D32" s="12">
-        <f>PPMT($B$4/12,A32,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A32,Months,-Amount)</f>
         <v>338.73923383565426</v>
       </c>
       <c r="E32" s="12">
@@ -1761,11 +1791,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C33" s="8">
-        <f>IPMT($B$4/12,A33,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A33,Months,-Amount)</f>
         <v>16.953587777975997</v>
       </c>
       <c r="D33" s="8">
-        <f>PPMT($B$4/12,A33,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A33,Months,-Amount)</f>
         <v>340.00950596253796</v>
       </c>
       <c r="E33" s="8">
@@ -1782,11 +1812,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C34" s="12">
-        <f>IPMT($B$4/12,A34,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A34,Months,-Amount)</f>
         <v>15.678552130616518</v>
       </c>
       <c r="D34" s="12">
-        <f>PPMT($B$4/12,A34,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A34,Months,-Amount)</f>
         <v>341.28454160989742</v>
       </c>
       <c r="E34" s="12">
@@ -1803,11 +1833,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C35" s="8">
-        <f>IPMT($B$4/12,A35,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A35,Months,-Amount)</f>
         <v>14.398735099579412</v>
       </c>
       <c r="D35" s="8">
-        <f>PPMT($B$4/12,A35,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A35,Months,-Amount)</f>
         <v>342.56435864093453</v>
       </c>
       <c r="E35" s="8">
@@ -1824,11 +1854,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C36" s="12">
-        <f>IPMT($B$4/12,A36,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A36,Months,-Amount)</f>
         <v>13.114118754675912</v>
       </c>
       <c r="D36" s="12">
-        <f>PPMT($B$4/12,A36,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A36,Months,-Amount)</f>
         <v>343.84897498583803</v>
       </c>
       <c r="E36" s="12">
@@ -1845,11 +1875,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C37" s="8">
-        <f>IPMT($B$4/12,A37,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A37,Months,-Amount)</f>
         <v>11.824685098479053</v>
       </c>
       <c r="D37" s="8">
-        <f>PPMT($B$4/12,A37,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A37,Months,-Amount)</f>
         <v>345.1384086420349</v>
       </c>
       <c r="E37" s="8">
@@ -1866,11 +1896,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C38" s="12">
-        <f>IPMT($B$4/12,A38,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A38,Months,-Amount)</f>
         <v>10.530416066071497</v>
       </c>
       <c r="D38" s="12">
-        <f>PPMT($B$4/12,A38,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A38,Months,-Amount)</f>
         <v>346.43267767444246</v>
       </c>
       <c r="E38" s="12">
@@ -1887,11 +1917,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C39" s="8">
-        <f>IPMT($B$4/12,A39,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A39,Months,-Amount)</f>
         <v>9.2312935247923402</v>
       </c>
       <c r="D39" s="8">
-        <f>PPMT($B$4/12,A39,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A39,Months,-Amount)</f>
         <v>347.73180021572159</v>
       </c>
       <c r="E39" s="8">
@@ -1908,11 +1938,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C40" s="12">
-        <f>IPMT($B$4/12,A40,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A40,Months,-Amount)</f>
         <v>7.9272992739834143</v>
       </c>
       <c r="D40" s="12">
-        <f>PPMT($B$4/12,A40,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A40,Months,-Amount)</f>
         <v>349.03579446653055</v>
       </c>
       <c r="E40" s="12">
@@ -1929,11 +1959,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C41" s="8">
-        <f>IPMT($B$4/12,A41,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A41,Months,-Amount)</f>
         <v>6.6184150447339398</v>
       </c>
       <c r="D41" s="8">
-        <f>PPMT($B$4/12,A41,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A41,Months,-Amount)</f>
         <v>350.34467869578003</v>
       </c>
       <c r="E41" s="8">
@@ -1950,11 +1980,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C42" s="12">
-        <f>IPMT($B$4/12,A42,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A42,Months,-Amount)</f>
         <v>5.3046224996248359</v>
       </c>
       <c r="D42" s="12">
-        <f>PPMT($B$4/12,A42,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A42,Months,-Amount)</f>
         <v>351.65847124088913</v>
       </c>
       <c r="E42" s="12">
@@ -1971,11 +2001,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C43" s="8">
-        <f>IPMT($B$4/12,A43,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A43,Months,-Amount)</f>
         <v>3.9859032324714803</v>
       </c>
       <c r="D43" s="8">
-        <f>PPMT($B$4/12,A43,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A43,Months,-Amount)</f>
         <v>352.9771905080425</v>
       </c>
       <c r="E43" s="8">
@@ -1992,11 +2022,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C44" s="12">
-        <f>IPMT($B$4/12,A44,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A44,Months,-Amount)</f>
         <v>2.6622387680663584</v>
       </c>
       <c r="D44" s="12">
-        <f>PPMT($B$4/12,A44,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A44,Months,-Amount)</f>
         <v>354.30085497244761</v>
       </c>
       <c r="E44" s="12">
@@ -2013,11 +2043,11 @@
         <v>356.96309374051395</v>
       </c>
       <c r="C45" s="8">
-        <f>IPMT($B$4/12,A45,$B$5,-$B$3)</f>
+        <f>IPMT(Rate/12,A45,Months,-Amount)</f>
         <v>1.3336105619197156</v>
       </c>
       <c r="D45" s="8">
-        <f>PPMT($B$4/12,A45,$B$5,-$B$3)</f>
+        <f>PPMT(Rate/12,A45,Months,-Amount)</f>
         <v>355.62948317859423</v>
       </c>
       <c r="E45" s="8">
@@ -2029,6 +2059,16 @@
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
+  <conditionalFormatting sqref="C10:C45">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>